<commit_message>
Added Collect Judgment from a Bank or Employer Easy Form to spreadsheet list
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ilao_docassemble_easy_forms.xlsx
+++ b/docassemble/ILAO/data/sources/ilao_docassemble_easy_forms.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VivianM\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B88F28DB-BA70-47F2-B161-683459368F05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4006083B-9E0E-4B81-B167-05E39FB0F928}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1884" yWindow="1884" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="110">
   <si>
     <t>name</t>
   </si>
@@ -349,6 +349,12 @@
   </si>
   <si>
     <t>Voluntary acknowledgment of parentage - VAP</t>
+  </si>
+  <si>
+    <t>Collect a judgment from debtor’s bank or employer</t>
+  </si>
+  <si>
+    <t>https://www.illinoislegalaid.org/legal-information/collect-judgment-debtors-bank-or-employer</t>
   </si>
 </sst>
 </file>
@@ -711,7 +717,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B54"/>
+  <dimension ref="A1:B55"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="44.5546875" bestFit="1" customWidth="1"/>
@@ -768,431 +774,439 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>108</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>71</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>91</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>84</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>22</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>103</v>
+        <v>21</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>104</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>58</v>
+        <v>103</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>59</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>4</v>
+        <v>58</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>7</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>55</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>3</v>
+        <v>54</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>6</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>72</v>
+        <v>3</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>73</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>10</v>
+        <v>72</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>11</v>
+        <v>73</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>106</v>
+        <v>30</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>105</v>
+        <v>32</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>25</v>
+        <v>106</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>83</v>
+        <v>31</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>82</v>
+        <v>33</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>50</v>
+        <v>83</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>51</v>
+        <v>82</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>86</v>
+        <v>48</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>87</v>
+        <v>49</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>44</v>
+        <v>86</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>45</v>
+        <v>87</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>65</v>
+        <v>47</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>16</v>
+        <v>65</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>79</v>
+        <v>16</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>99</v>
+        <v>79</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>27</v>
+        <v>98</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>28</v>
+        <v>99</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>74</v>
+        <v>27</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>9</v>
+        <v>68</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>8</v>
+        <v>69</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>61</v>
+        <v>9</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>60</v>
+        <v>8</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>14</v>
+        <v>76</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>15</v>
+        <v>77</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>96</v>
+        <v>34</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>97</v>
+        <v>35</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>81</v>
+        <v>102</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
+        <v>78</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
         <v>107</v>
       </c>
-      <c r="B54" s="1" t="s">
+      <c r="B55" s="1" t="s">
         <v>29</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B19">
-    <sortCondition ref="A2:A19"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B20">
+    <sortCondition ref="A2:A20"/>
   </sortState>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="B19" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="B16" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="B45" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="B21" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="B49" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="B38" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="B11" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="B12" r:id="rId9" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="B13" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="B41" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="B54" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="B22" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="B25" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="B50" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="B34" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="B35" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="B33" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="B32" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="B29" r:id="rId20" xr:uid="{E91D49D0-8A8A-49A5-B571-1E3A551885E4}"/>
-    <hyperlink ref="B27" r:id="rId21" xr:uid="{5EB32812-DDAD-43E1-BEC1-0E8706BB78F8}"/>
+    <hyperlink ref="B20" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="B17" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="B46" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="B22" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="B50" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="B39" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="B12" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="B13" r:id="rId9" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="B14" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="B42" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="B55" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="B23" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="B26" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="B51" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="B35" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="B36" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="B34" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="B33" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="B30" r:id="rId20" xr:uid="{E91D49D0-8A8A-49A5-B571-1E3A551885E4}"/>
+    <hyperlink ref="B28" r:id="rId21" xr:uid="{5EB32812-DDAD-43E1-BEC1-0E8706BB78F8}"/>
     <hyperlink ref="B4" r:id="rId22" xr:uid="{A23C6535-E02D-4241-B7AA-C698CCDB6D31}"/>
-    <hyperlink ref="B15" r:id="rId23" xr:uid="{5B0358E0-6FC3-4AF8-8E25-62EBF7059C1A}"/>
-    <hyperlink ref="B46" r:id="rId24" xr:uid="{1BD2E9FF-F69E-4E59-ACA9-BD41D2D4AE94}"/>
-    <hyperlink ref="B37" r:id="rId25" xr:uid="{620FD2E8-C9D1-4C14-8ED5-17B01AA5DA33}"/>
-    <hyperlink ref="B43" r:id="rId26" xr:uid="{226D490B-4537-4CB5-95DA-F750E9A0919D}"/>
-    <hyperlink ref="B47" r:id="rId27" xr:uid="{285D1364-5954-4A82-B493-EE664C0786D1}"/>
-    <hyperlink ref="B44" r:id="rId28" xr:uid="{BD0F8AFC-EDD1-4D31-AD59-8FAD5E6F7758}"/>
-    <hyperlink ref="B7" r:id="rId29" xr:uid="{4EAFCFFB-67EF-4EA4-9306-448CF1D5D183}"/>
-    <hyperlink ref="B20" r:id="rId30" xr:uid="{B1E55B86-EC01-47AD-AA8B-FA1792695821}"/>
-    <hyperlink ref="B39" r:id="rId31" xr:uid="{7A05A07A-CD46-49E0-8CAA-F7A2359DAFA6}"/>
-    <hyperlink ref="B53" r:id="rId32" xr:uid="{E8243C89-C7E6-4F98-8AB2-6F1F40304356}"/>
-    <hyperlink ref="B26" r:id="rId33" xr:uid="{A702F17D-AC4F-43CE-B44D-BF0EB0BA16F4}"/>
-    <hyperlink ref="B8" r:id="rId34" xr:uid="{A79B08AB-EC87-4B3E-B1A5-DB2982598670}"/>
-    <hyperlink ref="B51" r:id="rId35" xr:uid="{ACF5336B-7760-4E17-AB95-B490DF08E9B7}"/>
-    <hyperlink ref="B40" r:id="rId36" xr:uid="{5B5F40DA-F64F-4CBD-A95F-EBC3267FFA16}"/>
-    <hyperlink ref="B52" r:id="rId37" xr:uid="{CE808D58-61B9-423B-AD81-E68A94792CFB}"/>
-    <hyperlink ref="B23" r:id="rId38" xr:uid="{F1297A01-61E3-4759-9D5D-D9A6F9BCB77E}"/>
+    <hyperlink ref="B16" r:id="rId23" xr:uid="{5B0358E0-6FC3-4AF8-8E25-62EBF7059C1A}"/>
+    <hyperlink ref="B47" r:id="rId24" xr:uid="{1BD2E9FF-F69E-4E59-ACA9-BD41D2D4AE94}"/>
+    <hyperlink ref="B38" r:id="rId25" xr:uid="{620FD2E8-C9D1-4C14-8ED5-17B01AA5DA33}"/>
+    <hyperlink ref="B44" r:id="rId26" xr:uid="{226D490B-4537-4CB5-95DA-F750E9A0919D}"/>
+    <hyperlink ref="B48" r:id="rId27" xr:uid="{285D1364-5954-4A82-B493-EE664C0786D1}"/>
+    <hyperlink ref="B45" r:id="rId28" xr:uid="{BD0F8AFC-EDD1-4D31-AD59-8FAD5E6F7758}"/>
+    <hyperlink ref="B8" r:id="rId29" xr:uid="{4EAFCFFB-67EF-4EA4-9306-448CF1D5D183}"/>
+    <hyperlink ref="B21" r:id="rId30" xr:uid="{B1E55B86-EC01-47AD-AA8B-FA1792695821}"/>
+    <hyperlink ref="B40" r:id="rId31" xr:uid="{7A05A07A-CD46-49E0-8CAA-F7A2359DAFA6}"/>
+    <hyperlink ref="B54" r:id="rId32" xr:uid="{E8243C89-C7E6-4F98-8AB2-6F1F40304356}"/>
+    <hyperlink ref="B27" r:id="rId33" xr:uid="{A702F17D-AC4F-43CE-B44D-BF0EB0BA16F4}"/>
+    <hyperlink ref="B9" r:id="rId34" xr:uid="{A79B08AB-EC87-4B3E-B1A5-DB2982598670}"/>
+    <hyperlink ref="B52" r:id="rId35" xr:uid="{ACF5336B-7760-4E17-AB95-B490DF08E9B7}"/>
+    <hyperlink ref="B41" r:id="rId36" xr:uid="{5B5F40DA-F64F-4CBD-A95F-EBC3267FFA16}"/>
+    <hyperlink ref="B53" r:id="rId37" xr:uid="{CE808D58-61B9-423B-AD81-E68A94792CFB}"/>
+    <hyperlink ref="B24" r:id="rId38" xr:uid="{F1297A01-61E3-4759-9D5D-D9A6F9BCB77E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated framework to handle including English/Spanish support.
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ilao_docassemble_easy_forms.xlsx
+++ b/docassemble/ILAO/data/sources/ilao_docassemble_easy_forms.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\docassemble-ILAO\docassemble\ILAO\data\sources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC40A0F1-FAD3-4FF9-B622-655BE620B087}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D4F6E0F-51A2-4D42-AE9F-EAA6D144BFC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-34425" yWindow="-2655" windowWidth="30840" windowHeight="17085" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1610" yWindow="7330" windowWidth="30770" windowHeight="12300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,15 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="162">
   <si>
     <t>name</t>
   </si>
@@ -349,6 +352,168 @@
   </si>
   <si>
     <t>Joint simplified divorce - Cook County</t>
+  </si>
+  <si>
+    <t>name_es</t>
+  </si>
+  <si>
+    <t>Apariencia</t>
+  </si>
+  <si>
+    <t>Apariencia con presentación electrónica</t>
+  </si>
+  <si>
+    <t>Anulación de antecedentes penales por cannabis</t>
+  </si>
+  <si>
+    <t>Citación para descubrir bienes del deudor</t>
+  </si>
+  <si>
+    <t>Orden civil de no contacto - CNCO</t>
+  </si>
+  <si>
+    <t>Exención de cuotas judiciales penales</t>
+  </si>
+  <si>
+    <t>Carta a cobrador de deudas</t>
+  </si>
+  <si>
+    <t>Retrasar una venta por ejecución hipotecaria</t>
+  </si>
+  <si>
+    <t>Divorcio</t>
+  </si>
+  <si>
+    <t>Exención de presentación electrónica</t>
+  </si>
+  <si>
+    <t>Exención de presentación electrónica - Corte de Apelaciones</t>
+  </si>
+  <si>
+    <t>Exención de presentación electrónica - Corte Suprema</t>
+  </si>
+  <si>
+    <t>Moción de emergencia para reclamar exención</t>
+  </si>
+  <si>
+    <t>Orden de protección de emergencia - Condado de Cook</t>
+  </si>
+  <si>
+    <t>Carta para terminar bloqueo</t>
+  </si>
+  <si>
+    <t>Desalojar a un inquilino</t>
+  </si>
+  <si>
+    <t>Extender el tiempo de desalojo</t>
+  </si>
+  <si>
+    <t>Exención de cuotas</t>
+  </si>
+  <si>
+    <t>Declaración financiera</t>
+  </si>
+  <si>
+    <t>Queja por discriminación de vivienda - IDHR</t>
+  </si>
+  <si>
+    <t>Solicitud de intérprete</t>
+  </si>
+  <si>
+    <t>Divorcio simplificado conjunto - Condado de Cook</t>
+  </si>
+  <si>
+    <t>Testamento vital</t>
+  </si>
+  <si>
+    <t>Moción</t>
+  </si>
+  <si>
+    <t>Moción para continuar o extender el tiempo</t>
+  </si>
+  <si>
+    <t>Cambio de nombre para un adulto</t>
+  </si>
+  <si>
+    <t>Cambio de nombre para un menor</t>
+  </si>
+  <si>
+    <t>Orden de protección</t>
+  </si>
+  <si>
+    <t>Plan de crianza</t>
+  </si>
+  <si>
+    <t>Solicitud de archivo de personal</t>
+  </si>
+  <si>
+    <t>Poder notarial para cuidado de la salud</t>
+  </si>
+  <si>
+    <t>Poder notarial para propiedad</t>
+  </si>
+  <si>
+    <t>Renuncia de poder notarial</t>
+  </si>
+  <si>
+    <t>Revocación de poder notarial</t>
+  </si>
+  <si>
+    <t>Comprobante de entrega</t>
+  </si>
+  <si>
+    <t>Eliminar desalojo del registro público</t>
+  </si>
+  <si>
+    <t>Solicitud de tiempo libre después de sobrevivir violencia</t>
+  </si>
+  <si>
+    <t>Solicitud para aprobar un servidor de procesos sin licencia</t>
+  </si>
+  <si>
+    <t>Solicitud para cambiar manutención infantil</t>
+  </si>
+  <si>
+    <t>Responder a una demanda</t>
+  </si>
+  <si>
+    <t>Responder a una queja de ejecución hipotecaria</t>
+  </si>
+  <si>
+    <t>Responder a un desalojo</t>
+  </si>
+  <si>
+    <t>Queja por depósito de seguridad</t>
+  </si>
+  <si>
+    <t>Carta de demanda de depósito de seguridad</t>
+  </si>
+  <si>
+    <t>Tutela a corto plazo</t>
+  </si>
+  <si>
+    <t>Demanda en tribunales de lo menor</t>
+  </si>
+  <si>
+    <t>Orden de no contacto por acoso - SNCO</t>
+  </si>
+  <si>
+    <t>Detener asignación de salario</t>
+  </si>
+  <si>
+    <t>Instrumento de transferencia por muerte - TODI</t>
+  </si>
+  <si>
+    <t>Solicitud de audiencia para prestaciones de desempleo</t>
+  </si>
+  <si>
+    <t>Anular sentencia por incumplimiento en ejecución hipotecaria</t>
+  </si>
+  <si>
+    <t>Anular sentencia por incumplimiento dentro de 30 días</t>
+  </si>
+  <si>
+    <t>Reconocimiento voluntario de paternidad - VAP</t>
   </si>
 </sst>
 </file>
@@ -711,443 +876,606 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B54"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C54"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="44.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="104.44140625" customWidth="1"/>
+    <col min="1" max="1" width="44.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="104.453125" customWidth="1"/>
+    <col min="3" max="3" width="59.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>17</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>53</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>95</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>93</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C6" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>71</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C7" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>91</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>89</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C9" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>85</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C10" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>19</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C11" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>20</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>21</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C13" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>104</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C14" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>59</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C15" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>4</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C16" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>12</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C17" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>55</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C18" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>3</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C19" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>73</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C20" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>10</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C21" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>31</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C22" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>107</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C23" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>25</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C24" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>32</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C25" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>84</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C26" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>51</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C27" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>57</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C28" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>49</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C29" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>87</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C30" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>45</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C31" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>43</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C32" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>41</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C33" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>38</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C34" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>39</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C35" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>47</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C36" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>64</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C37" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>101</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C38" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>81</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C39" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>99</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C40" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>27</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C41" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>75</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C42" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>63</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C43" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>69</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C44" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>9</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C45" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>62</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C46" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>65</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C47" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>77</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C48" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>14</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C49" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>35</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C50" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>97</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C51" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>102</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C52" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>79</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C53" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>29</v>
       </c>
       <c r="B54" s="1" t="s">
         <v>30</v>
+      </c>
+      <c r="C54" t="s">
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -1195,5 +1523,6 @@
     <hyperlink ref="B23" r:id="rId38" xr:uid="{F1297A01-61E3-4759-9D5D-D9A6F9BCB77E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added minor guardianship to xlsx
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ilao_docassemble_easy_forms.xlsx
+++ b/docassemble/ILAO/data/sources/ilao_docassemble_easy_forms.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VivianM\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4006083B-9E0E-4B81-B167-05E39FB0F928}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5618CC0-8E9B-4D34-82B9-56E314852436}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25455" yWindow="-4095" windowWidth="22575" windowHeight="15540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="112">
   <si>
     <t>name</t>
   </si>
@@ -355,6 +355,12 @@
   </si>
   <si>
     <t>https://www.illinoislegalaid.org/legal-information/collect-judgment-debtors-bank-or-employer</t>
+  </si>
+  <si>
+    <t>Guardianship of a child</t>
+  </si>
+  <si>
+    <t>https://www.illinoislegalaid.org/legal-information/guardianship-child</t>
   </si>
 </sst>
 </file>
@@ -717,7 +723,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B55"/>
+  <dimension ref="A1:B56"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="44.5546875" bestFit="1" customWidth="1"/>
@@ -894,273 +900,281 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>10</v>
+        <v>110</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>11</v>
+        <v>111</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>106</v>
+        <v>30</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>105</v>
+        <v>32</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>25</v>
+        <v>106</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>83</v>
+        <v>31</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>82</v>
+        <v>33</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>50</v>
+        <v>83</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>51</v>
+        <v>82</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>86</v>
+        <v>48</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>87</v>
+        <v>49</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>44</v>
+        <v>86</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>45</v>
+        <v>87</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>65</v>
+        <v>47</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>16</v>
+        <v>65</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>79</v>
+        <v>16</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>99</v>
+        <v>79</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>27</v>
+        <v>98</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>28</v>
+        <v>99</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>74</v>
+        <v>27</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>9</v>
+        <v>68</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>8</v>
+        <v>69</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>61</v>
+        <v>9</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>60</v>
+        <v>8</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>14</v>
+        <v>76</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>15</v>
+        <v>77</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>96</v>
+        <v>34</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>97</v>
+        <v>35</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>81</v>
+        <v>102</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
+        <v>78</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
         <v>107</v>
       </c>
-      <c r="B55" s="1" t="s">
+      <c r="B56" s="1" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1172,41 +1186,42 @@
     <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="B20" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="B17" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="B46" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="B22" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="B50" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="B39" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="B47" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="B23" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="B51" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="B40" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
     <hyperlink ref="B12" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
     <hyperlink ref="B13" r:id="rId9" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
     <hyperlink ref="B14" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="B42" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="B55" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="B23" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="B26" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="B51" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="B35" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="B36" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="B34" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="B33" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="B30" r:id="rId20" xr:uid="{E91D49D0-8A8A-49A5-B571-1E3A551885E4}"/>
-    <hyperlink ref="B28" r:id="rId21" xr:uid="{5EB32812-DDAD-43E1-BEC1-0E8706BB78F8}"/>
+    <hyperlink ref="B43" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="B56" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="B24" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="B27" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="B52" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="B36" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="B37" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="B35" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="B34" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="B31" r:id="rId20" xr:uid="{E91D49D0-8A8A-49A5-B571-1E3A551885E4}"/>
+    <hyperlink ref="B29" r:id="rId21" xr:uid="{5EB32812-DDAD-43E1-BEC1-0E8706BB78F8}"/>
     <hyperlink ref="B4" r:id="rId22" xr:uid="{A23C6535-E02D-4241-B7AA-C698CCDB6D31}"/>
     <hyperlink ref="B16" r:id="rId23" xr:uid="{5B0358E0-6FC3-4AF8-8E25-62EBF7059C1A}"/>
-    <hyperlink ref="B47" r:id="rId24" xr:uid="{1BD2E9FF-F69E-4E59-ACA9-BD41D2D4AE94}"/>
-    <hyperlink ref="B38" r:id="rId25" xr:uid="{620FD2E8-C9D1-4C14-8ED5-17B01AA5DA33}"/>
-    <hyperlink ref="B44" r:id="rId26" xr:uid="{226D490B-4537-4CB5-95DA-F750E9A0919D}"/>
-    <hyperlink ref="B48" r:id="rId27" xr:uid="{285D1364-5954-4A82-B493-EE664C0786D1}"/>
-    <hyperlink ref="B45" r:id="rId28" xr:uid="{BD0F8AFC-EDD1-4D31-AD59-8FAD5E6F7758}"/>
+    <hyperlink ref="B48" r:id="rId24" xr:uid="{1BD2E9FF-F69E-4E59-ACA9-BD41D2D4AE94}"/>
+    <hyperlink ref="B39" r:id="rId25" xr:uid="{620FD2E8-C9D1-4C14-8ED5-17B01AA5DA33}"/>
+    <hyperlink ref="B45" r:id="rId26" xr:uid="{226D490B-4537-4CB5-95DA-F750E9A0919D}"/>
+    <hyperlink ref="B49" r:id="rId27" xr:uid="{285D1364-5954-4A82-B493-EE664C0786D1}"/>
+    <hyperlink ref="B46" r:id="rId28" xr:uid="{BD0F8AFC-EDD1-4D31-AD59-8FAD5E6F7758}"/>
     <hyperlink ref="B8" r:id="rId29" xr:uid="{4EAFCFFB-67EF-4EA4-9306-448CF1D5D183}"/>
     <hyperlink ref="B21" r:id="rId30" xr:uid="{B1E55B86-EC01-47AD-AA8B-FA1792695821}"/>
-    <hyperlink ref="B40" r:id="rId31" xr:uid="{7A05A07A-CD46-49E0-8CAA-F7A2359DAFA6}"/>
-    <hyperlink ref="B54" r:id="rId32" xr:uid="{E8243C89-C7E6-4F98-8AB2-6F1F40304356}"/>
-    <hyperlink ref="B27" r:id="rId33" xr:uid="{A702F17D-AC4F-43CE-B44D-BF0EB0BA16F4}"/>
+    <hyperlink ref="B41" r:id="rId31" xr:uid="{7A05A07A-CD46-49E0-8CAA-F7A2359DAFA6}"/>
+    <hyperlink ref="B55" r:id="rId32" xr:uid="{E8243C89-C7E6-4F98-8AB2-6F1F40304356}"/>
+    <hyperlink ref="B28" r:id="rId33" xr:uid="{A702F17D-AC4F-43CE-B44D-BF0EB0BA16F4}"/>
     <hyperlink ref="B9" r:id="rId34" xr:uid="{A79B08AB-EC87-4B3E-B1A5-DB2982598670}"/>
-    <hyperlink ref="B52" r:id="rId35" xr:uid="{ACF5336B-7760-4E17-AB95-B490DF08E9B7}"/>
-    <hyperlink ref="B41" r:id="rId36" xr:uid="{5B5F40DA-F64F-4CBD-A95F-EBC3267FFA16}"/>
-    <hyperlink ref="B53" r:id="rId37" xr:uid="{CE808D58-61B9-423B-AD81-E68A94792CFB}"/>
-    <hyperlink ref="B24" r:id="rId38" xr:uid="{F1297A01-61E3-4759-9D5D-D9A6F9BCB77E}"/>
+    <hyperlink ref="B53" r:id="rId35" xr:uid="{ACF5336B-7760-4E17-AB95-B490DF08E9B7}"/>
+    <hyperlink ref="B42" r:id="rId36" xr:uid="{5B5F40DA-F64F-4CBD-A95F-EBC3267FFA16}"/>
+    <hyperlink ref="B54" r:id="rId37" xr:uid="{CE808D58-61B9-423B-AD81-E68A94792CFB}"/>
+    <hyperlink ref="B25" r:id="rId38" xr:uid="{F1297A01-61E3-4759-9D5D-D9A6F9BCB77E}"/>
+    <hyperlink ref="B22" r:id="rId39" xr:uid="{C745FACC-7FAC-461E-90D4-9BC0A4025913}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added Rental repair letter to easy forms xlsx
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ilao_docassemble_easy_forms.xlsx
+++ b/docassemble/ILAO/data/sources/ilao_docassemble_easy_forms.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VivianM\Desktop\Easy Forms\Rental Repair Letter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5618CC0-8E9B-4D34-82B9-56E314852436}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E383E5F9-9754-4285-902B-8FB9EE22D0B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25455" yWindow="-4095" windowWidth="22575" windowHeight="15540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="114">
   <si>
     <t>name</t>
   </si>
@@ -361,6 +361,12 @@
   </si>
   <si>
     <t>https://www.illinoislegalaid.org/legal-information/guardianship-child</t>
+  </si>
+  <si>
+    <t>Rental repair letter</t>
+  </si>
+  <si>
+    <t>https://www.illinoislegalaid.org/legal-information/rental-repair-letter</t>
   </si>
 </sst>
 </file>
@@ -723,7 +729,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B56"/>
+  <dimension ref="A1:B57"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="44.5546875" bestFit="1" customWidth="1"/>
@@ -1044,137 +1050,145 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>16</v>
+        <v>113</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>79</v>
+        <v>16</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>99</v>
+        <v>79</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>27</v>
+        <v>98</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>28</v>
+        <v>99</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>74</v>
+        <v>27</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>9</v>
+        <v>68</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>8</v>
+        <v>69</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>61</v>
+        <v>9</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>60</v>
+        <v>8</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>14</v>
+        <v>76</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>15</v>
+        <v>77</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>96</v>
+        <v>34</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>97</v>
+        <v>35</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>81</v>
+        <v>102</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
+        <v>78</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
         <v>107</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B57" s="1" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1186,42 +1200,43 @@
     <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="B20" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="B17" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="B47" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="B48" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
     <hyperlink ref="B23" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="B51" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="B40" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="B52" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="B41" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
     <hyperlink ref="B12" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
     <hyperlink ref="B13" r:id="rId9" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
     <hyperlink ref="B14" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="B43" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="B56" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="B24" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="B27" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="B52" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="B36" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="B37" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="B35" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="B34" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="B31" r:id="rId20" xr:uid="{E91D49D0-8A8A-49A5-B571-1E3A551885E4}"/>
-    <hyperlink ref="B29" r:id="rId21" xr:uid="{5EB32812-DDAD-43E1-BEC1-0E8706BB78F8}"/>
-    <hyperlink ref="B4" r:id="rId22" xr:uid="{A23C6535-E02D-4241-B7AA-C698CCDB6D31}"/>
-    <hyperlink ref="B16" r:id="rId23" xr:uid="{5B0358E0-6FC3-4AF8-8E25-62EBF7059C1A}"/>
-    <hyperlink ref="B48" r:id="rId24" xr:uid="{1BD2E9FF-F69E-4E59-ACA9-BD41D2D4AE94}"/>
-    <hyperlink ref="B39" r:id="rId25" xr:uid="{620FD2E8-C9D1-4C14-8ED5-17B01AA5DA33}"/>
-    <hyperlink ref="B45" r:id="rId26" xr:uid="{226D490B-4537-4CB5-95DA-F750E9A0919D}"/>
-    <hyperlink ref="B49" r:id="rId27" xr:uid="{285D1364-5954-4A82-B493-EE664C0786D1}"/>
-    <hyperlink ref="B46" r:id="rId28" xr:uid="{BD0F8AFC-EDD1-4D31-AD59-8FAD5E6F7758}"/>
-    <hyperlink ref="B8" r:id="rId29" xr:uid="{4EAFCFFB-67EF-4EA4-9306-448CF1D5D183}"/>
-    <hyperlink ref="B21" r:id="rId30" xr:uid="{B1E55B86-EC01-47AD-AA8B-FA1792695821}"/>
-    <hyperlink ref="B41" r:id="rId31" xr:uid="{7A05A07A-CD46-49E0-8CAA-F7A2359DAFA6}"/>
-    <hyperlink ref="B55" r:id="rId32" xr:uid="{E8243C89-C7E6-4F98-8AB2-6F1F40304356}"/>
-    <hyperlink ref="B28" r:id="rId33" xr:uid="{A702F17D-AC4F-43CE-B44D-BF0EB0BA16F4}"/>
-    <hyperlink ref="B9" r:id="rId34" xr:uid="{A79B08AB-EC87-4B3E-B1A5-DB2982598670}"/>
-    <hyperlink ref="B53" r:id="rId35" xr:uid="{ACF5336B-7760-4E17-AB95-B490DF08E9B7}"/>
-    <hyperlink ref="B42" r:id="rId36" xr:uid="{5B5F40DA-F64F-4CBD-A95F-EBC3267FFA16}"/>
-    <hyperlink ref="B54" r:id="rId37" xr:uid="{CE808D58-61B9-423B-AD81-E68A94792CFB}"/>
-    <hyperlink ref="B25" r:id="rId38" xr:uid="{F1297A01-61E3-4759-9D5D-D9A6F9BCB77E}"/>
-    <hyperlink ref="B22" r:id="rId39" xr:uid="{C745FACC-7FAC-461E-90D4-9BC0A4025913}"/>
+    <hyperlink ref="B44" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="B24" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="B27" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="B53" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="B36" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="B37" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="B35" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="B34" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="B31" r:id="rId19" xr:uid="{E91D49D0-8A8A-49A5-B571-1E3A551885E4}"/>
+    <hyperlink ref="B29" r:id="rId20" xr:uid="{5EB32812-DDAD-43E1-BEC1-0E8706BB78F8}"/>
+    <hyperlink ref="B4" r:id="rId21" xr:uid="{A23C6535-E02D-4241-B7AA-C698CCDB6D31}"/>
+    <hyperlink ref="B16" r:id="rId22" xr:uid="{5B0358E0-6FC3-4AF8-8E25-62EBF7059C1A}"/>
+    <hyperlink ref="B49" r:id="rId23" xr:uid="{1BD2E9FF-F69E-4E59-ACA9-BD41D2D4AE94}"/>
+    <hyperlink ref="B39" r:id="rId24" xr:uid="{620FD2E8-C9D1-4C14-8ED5-17B01AA5DA33}"/>
+    <hyperlink ref="B46" r:id="rId25" xr:uid="{226D490B-4537-4CB5-95DA-F750E9A0919D}"/>
+    <hyperlink ref="B50" r:id="rId26" xr:uid="{285D1364-5954-4A82-B493-EE664C0786D1}"/>
+    <hyperlink ref="B47" r:id="rId27" xr:uid="{BD0F8AFC-EDD1-4D31-AD59-8FAD5E6F7758}"/>
+    <hyperlink ref="B8" r:id="rId28" xr:uid="{4EAFCFFB-67EF-4EA4-9306-448CF1D5D183}"/>
+    <hyperlink ref="B21" r:id="rId29" xr:uid="{B1E55B86-EC01-47AD-AA8B-FA1792695821}"/>
+    <hyperlink ref="B42" r:id="rId30" xr:uid="{7A05A07A-CD46-49E0-8CAA-F7A2359DAFA6}"/>
+    <hyperlink ref="B56" r:id="rId31" xr:uid="{E8243C89-C7E6-4F98-8AB2-6F1F40304356}"/>
+    <hyperlink ref="B28" r:id="rId32" xr:uid="{A702F17D-AC4F-43CE-B44D-BF0EB0BA16F4}"/>
+    <hyperlink ref="B9" r:id="rId33" xr:uid="{A79B08AB-EC87-4B3E-B1A5-DB2982598670}"/>
+    <hyperlink ref="B54" r:id="rId34" xr:uid="{ACF5336B-7760-4E17-AB95-B490DF08E9B7}"/>
+    <hyperlink ref="B43" r:id="rId35" xr:uid="{5B5F40DA-F64F-4CBD-A95F-EBC3267FFA16}"/>
+    <hyperlink ref="B55" r:id="rId36" xr:uid="{CE808D58-61B9-423B-AD81-E68A94792CFB}"/>
+    <hyperlink ref="B25" r:id="rId37" xr:uid="{F1297A01-61E3-4759-9D5D-D9A6F9BCB77E}"/>
+    <hyperlink ref="B22" r:id="rId38" xr:uid="{C745FACC-7FAC-461E-90D4-9BC0A4025913}"/>
+    <hyperlink ref="B57" r:id="rId39" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="B40" r:id="rId40" xr:uid="{19683C75-D4BA-4207-8A88-14E281FC0EF3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
unemployment appeal after hearing and appellate fee waiver
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ilao_docassemble_easy_forms.xlsx
+++ b/docassemble/ILAO/data/sources/ilao_docassemble_easy_forms.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VivianM\Desktop\Easy Forms\Rental Repair Letter\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E383E5F9-9754-4285-902B-8FB9EE22D0B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{914F1CB4-EC4A-447B-804D-AC159B0F1876}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-36720" yWindow="-3495" windowWidth="30570" windowHeight="17985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="118">
   <si>
     <t>name</t>
   </si>
@@ -367,6 +367,18 @@
   </si>
   <si>
     <t>https://www.illinoislegalaid.org/legal-information/rental-repair-letter</t>
+  </si>
+  <si>
+    <t>Fee waiver - Appellate Court</t>
+  </si>
+  <si>
+    <t>https://www.illinoislegalaid.org/legal-information/fee-waiver-appellate-court</t>
+  </si>
+  <si>
+    <t>Unemployment benefits appeal after a hearing</t>
+  </si>
+  <si>
+    <t>https://www.illinoislegalaid.org/legal-information/unemployment-benefits-appeal</t>
   </si>
 </sst>
 </file>
@@ -729,7 +741,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B57"/>
+  <dimension ref="A1:B59"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="44.5546875" bestFit="1" customWidth="1"/>
@@ -898,297 +910,313 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>72</v>
+        <v>114</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>73</v>
+        <v>115</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>110</v>
+        <v>72</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>111</v>
+        <v>73</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>10</v>
+        <v>110</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>11</v>
+        <v>111</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>106</v>
+        <v>30</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>105</v>
+        <v>32</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>25</v>
+        <v>106</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>83</v>
+        <v>31</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>82</v>
+        <v>33</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>50</v>
+        <v>83</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>51</v>
+        <v>82</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>86</v>
+        <v>48</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>87</v>
+        <v>49</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>44</v>
+        <v>86</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>45</v>
+        <v>87</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>65</v>
+        <v>47</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>112</v>
+        <v>63</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>113</v>
+        <v>65</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>16</v>
+        <v>113</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>79</v>
+        <v>16</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>99</v>
+        <v>79</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>27</v>
+        <v>98</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>28</v>
+        <v>99</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>74</v>
+        <v>27</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>9</v>
+        <v>68</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>8</v>
+        <v>69</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>61</v>
+        <v>9</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>60</v>
+        <v>8</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>14</v>
+        <v>76</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>15</v>
+        <v>77</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>96</v>
+        <v>34</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>97</v>
+        <v>35</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
+        <v>101</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>78</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
         <v>107</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="B59" s="1" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1200,43 +1228,45 @@
     <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="B20" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="B17" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="B48" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="B23" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="B52" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="B41" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="B49" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="B24" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="B53" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="B42" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
     <hyperlink ref="B12" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
     <hyperlink ref="B13" r:id="rId9" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
     <hyperlink ref="B14" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="B44" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="B24" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="B27" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="B53" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="B36" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="B37" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="B35" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="B34" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="B31" r:id="rId19" xr:uid="{E91D49D0-8A8A-49A5-B571-1E3A551885E4}"/>
-    <hyperlink ref="B29" r:id="rId20" xr:uid="{5EB32812-DDAD-43E1-BEC1-0E8706BB78F8}"/>
+    <hyperlink ref="B45" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="B25" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="B28" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="B54" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="B37" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="B38" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="B36" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="B35" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="B32" r:id="rId19" xr:uid="{E91D49D0-8A8A-49A5-B571-1E3A551885E4}"/>
+    <hyperlink ref="B30" r:id="rId20" xr:uid="{5EB32812-DDAD-43E1-BEC1-0E8706BB78F8}"/>
     <hyperlink ref="B4" r:id="rId21" xr:uid="{A23C6535-E02D-4241-B7AA-C698CCDB6D31}"/>
     <hyperlink ref="B16" r:id="rId22" xr:uid="{5B0358E0-6FC3-4AF8-8E25-62EBF7059C1A}"/>
-    <hyperlink ref="B49" r:id="rId23" xr:uid="{1BD2E9FF-F69E-4E59-ACA9-BD41D2D4AE94}"/>
-    <hyperlink ref="B39" r:id="rId24" xr:uid="{620FD2E8-C9D1-4C14-8ED5-17B01AA5DA33}"/>
-    <hyperlink ref="B46" r:id="rId25" xr:uid="{226D490B-4537-4CB5-95DA-F750E9A0919D}"/>
-    <hyperlink ref="B50" r:id="rId26" xr:uid="{285D1364-5954-4A82-B493-EE664C0786D1}"/>
-    <hyperlink ref="B47" r:id="rId27" xr:uid="{BD0F8AFC-EDD1-4D31-AD59-8FAD5E6F7758}"/>
+    <hyperlink ref="B50" r:id="rId23" xr:uid="{1BD2E9FF-F69E-4E59-ACA9-BD41D2D4AE94}"/>
+    <hyperlink ref="B40" r:id="rId24" xr:uid="{620FD2E8-C9D1-4C14-8ED5-17B01AA5DA33}"/>
+    <hyperlink ref="B47" r:id="rId25" xr:uid="{226D490B-4537-4CB5-95DA-F750E9A0919D}"/>
+    <hyperlink ref="B51" r:id="rId26" xr:uid="{285D1364-5954-4A82-B493-EE664C0786D1}"/>
+    <hyperlink ref="B48" r:id="rId27" xr:uid="{BD0F8AFC-EDD1-4D31-AD59-8FAD5E6F7758}"/>
     <hyperlink ref="B8" r:id="rId28" xr:uid="{4EAFCFFB-67EF-4EA4-9306-448CF1D5D183}"/>
-    <hyperlink ref="B21" r:id="rId29" xr:uid="{B1E55B86-EC01-47AD-AA8B-FA1792695821}"/>
-    <hyperlink ref="B42" r:id="rId30" xr:uid="{7A05A07A-CD46-49E0-8CAA-F7A2359DAFA6}"/>
-    <hyperlink ref="B56" r:id="rId31" xr:uid="{E8243C89-C7E6-4F98-8AB2-6F1F40304356}"/>
-    <hyperlink ref="B28" r:id="rId32" xr:uid="{A702F17D-AC4F-43CE-B44D-BF0EB0BA16F4}"/>
+    <hyperlink ref="B22" r:id="rId29" xr:uid="{B1E55B86-EC01-47AD-AA8B-FA1792695821}"/>
+    <hyperlink ref="B43" r:id="rId30" xr:uid="{7A05A07A-CD46-49E0-8CAA-F7A2359DAFA6}"/>
+    <hyperlink ref="B58" r:id="rId31" xr:uid="{E8243C89-C7E6-4F98-8AB2-6F1F40304356}"/>
+    <hyperlink ref="B29" r:id="rId32" xr:uid="{A702F17D-AC4F-43CE-B44D-BF0EB0BA16F4}"/>
     <hyperlink ref="B9" r:id="rId33" xr:uid="{A79B08AB-EC87-4B3E-B1A5-DB2982598670}"/>
-    <hyperlink ref="B54" r:id="rId34" xr:uid="{ACF5336B-7760-4E17-AB95-B490DF08E9B7}"/>
-    <hyperlink ref="B43" r:id="rId35" xr:uid="{5B5F40DA-F64F-4CBD-A95F-EBC3267FFA16}"/>
-    <hyperlink ref="B55" r:id="rId36" xr:uid="{CE808D58-61B9-423B-AD81-E68A94792CFB}"/>
-    <hyperlink ref="B25" r:id="rId37" xr:uid="{F1297A01-61E3-4759-9D5D-D9A6F9BCB77E}"/>
-    <hyperlink ref="B22" r:id="rId38" xr:uid="{C745FACC-7FAC-461E-90D4-9BC0A4025913}"/>
-    <hyperlink ref="B57" r:id="rId39" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="B40" r:id="rId40" xr:uid="{19683C75-D4BA-4207-8A88-14E281FC0EF3}"/>
+    <hyperlink ref="B56" r:id="rId34" xr:uid="{ACF5336B-7760-4E17-AB95-B490DF08E9B7}"/>
+    <hyperlink ref="B44" r:id="rId35" xr:uid="{5B5F40DA-F64F-4CBD-A95F-EBC3267FFA16}"/>
+    <hyperlink ref="B57" r:id="rId36" xr:uid="{CE808D58-61B9-423B-AD81-E68A94792CFB}"/>
+    <hyperlink ref="B26" r:id="rId37" xr:uid="{F1297A01-61E3-4759-9D5D-D9A6F9BCB77E}"/>
+    <hyperlink ref="B23" r:id="rId38" xr:uid="{C745FACC-7FAC-461E-90D4-9BC0A4025913}"/>
+    <hyperlink ref="B59" r:id="rId39" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="B41" r:id="rId40" xr:uid="{19683C75-D4BA-4207-8A88-14E281FC0EF3}"/>
+    <hyperlink ref="B21" r:id="rId41" xr:uid="{90E3F36C-96B8-4969-BD97-8904E85B3EC2}"/>
+    <hyperlink ref="B55" r:id="rId42" xr:uid="{C93BA389-85D0-4EED-A95D-B84989BC0704}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added Request property in car program to spreadsheet list
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ilao_docassemble_easy_forms.xlsx
+++ b/docassemble/ILAO/data/sources/ilao_docassemble_easy_forms.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VivianM\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{914F1CB4-EC4A-447B-804D-AC159B0F1876}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E111C3E7-F726-4DB1-BB52-B86D00C04FF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-36720" yWindow="-3495" windowWidth="30570" windowHeight="17985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="120">
   <si>
     <t>name</t>
   </si>
@@ -379,6 +379,12 @@
   </si>
   <si>
     <t>https://www.illinoislegalaid.org/legal-information/unemployment-benefits-appeal</t>
+  </si>
+  <si>
+    <t>Request for personal property left inside a repossessed car</t>
+  </si>
+  <si>
+    <t>https://www.illinoislegalaid.org/legal-information/request-personal-property-left-inside-repossessed-car</t>
   </si>
 </sst>
 </file>
@@ -741,10 +747,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B59"/>
+  <dimension ref="A1:B60"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="44.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="49.77734375" customWidth="1"/>
     <col min="2" max="2" width="104.44140625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1078,145 +1084,153 @@
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>100</v>
+        <v>118</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>16</v>
+        <v>119</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>79</v>
+        <v>16</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>99</v>
+        <v>79</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>27</v>
+        <v>98</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>28</v>
+        <v>99</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>74</v>
+        <v>27</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>9</v>
+        <v>68</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>8</v>
+        <v>69</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>61</v>
+        <v>9</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>60</v>
+        <v>8</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>14</v>
+        <v>76</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>15</v>
+        <v>77</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>116</v>
+        <v>34</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>117</v>
+        <v>35</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>96</v>
+        <v>116</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>97</v>
+        <v>117</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>81</v>
+        <v>102</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
+        <v>78</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
         <v>107</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="B60" s="1" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1228,17 +1242,17 @@
     <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="B20" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="B17" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="B49" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="B50" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
     <hyperlink ref="B24" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="B53" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="B42" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="B54" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="B43" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
     <hyperlink ref="B12" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
     <hyperlink ref="B13" r:id="rId9" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
     <hyperlink ref="B14" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="B45" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="B46" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
     <hyperlink ref="B25" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
     <hyperlink ref="B28" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="B54" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="B55" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
     <hyperlink ref="B37" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
     <hyperlink ref="B38" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
     <hyperlink ref="B36" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
@@ -1247,26 +1261,27 @@
     <hyperlink ref="B30" r:id="rId20" xr:uid="{5EB32812-DDAD-43E1-BEC1-0E8706BB78F8}"/>
     <hyperlink ref="B4" r:id="rId21" xr:uid="{A23C6535-E02D-4241-B7AA-C698CCDB6D31}"/>
     <hyperlink ref="B16" r:id="rId22" xr:uid="{5B0358E0-6FC3-4AF8-8E25-62EBF7059C1A}"/>
-    <hyperlink ref="B50" r:id="rId23" xr:uid="{1BD2E9FF-F69E-4E59-ACA9-BD41D2D4AE94}"/>
+    <hyperlink ref="B51" r:id="rId23" xr:uid="{1BD2E9FF-F69E-4E59-ACA9-BD41D2D4AE94}"/>
     <hyperlink ref="B40" r:id="rId24" xr:uid="{620FD2E8-C9D1-4C14-8ED5-17B01AA5DA33}"/>
-    <hyperlink ref="B47" r:id="rId25" xr:uid="{226D490B-4537-4CB5-95DA-F750E9A0919D}"/>
-    <hyperlink ref="B51" r:id="rId26" xr:uid="{285D1364-5954-4A82-B493-EE664C0786D1}"/>
-    <hyperlink ref="B48" r:id="rId27" xr:uid="{BD0F8AFC-EDD1-4D31-AD59-8FAD5E6F7758}"/>
+    <hyperlink ref="B48" r:id="rId25" xr:uid="{226D490B-4537-4CB5-95DA-F750E9A0919D}"/>
+    <hyperlink ref="B52" r:id="rId26" xr:uid="{285D1364-5954-4A82-B493-EE664C0786D1}"/>
+    <hyperlink ref="B49" r:id="rId27" xr:uid="{BD0F8AFC-EDD1-4D31-AD59-8FAD5E6F7758}"/>
     <hyperlink ref="B8" r:id="rId28" xr:uid="{4EAFCFFB-67EF-4EA4-9306-448CF1D5D183}"/>
     <hyperlink ref="B22" r:id="rId29" xr:uid="{B1E55B86-EC01-47AD-AA8B-FA1792695821}"/>
-    <hyperlink ref="B43" r:id="rId30" xr:uid="{7A05A07A-CD46-49E0-8CAA-F7A2359DAFA6}"/>
-    <hyperlink ref="B58" r:id="rId31" xr:uid="{E8243C89-C7E6-4F98-8AB2-6F1F40304356}"/>
+    <hyperlink ref="B44" r:id="rId30" xr:uid="{7A05A07A-CD46-49E0-8CAA-F7A2359DAFA6}"/>
+    <hyperlink ref="B59" r:id="rId31" xr:uid="{E8243C89-C7E6-4F98-8AB2-6F1F40304356}"/>
     <hyperlink ref="B29" r:id="rId32" xr:uid="{A702F17D-AC4F-43CE-B44D-BF0EB0BA16F4}"/>
     <hyperlink ref="B9" r:id="rId33" xr:uid="{A79B08AB-EC87-4B3E-B1A5-DB2982598670}"/>
-    <hyperlink ref="B56" r:id="rId34" xr:uid="{ACF5336B-7760-4E17-AB95-B490DF08E9B7}"/>
-    <hyperlink ref="B44" r:id="rId35" xr:uid="{5B5F40DA-F64F-4CBD-A95F-EBC3267FFA16}"/>
-    <hyperlink ref="B57" r:id="rId36" xr:uid="{CE808D58-61B9-423B-AD81-E68A94792CFB}"/>
+    <hyperlink ref="B57" r:id="rId34" xr:uid="{ACF5336B-7760-4E17-AB95-B490DF08E9B7}"/>
+    <hyperlink ref="B45" r:id="rId35" xr:uid="{5B5F40DA-F64F-4CBD-A95F-EBC3267FFA16}"/>
+    <hyperlink ref="B58" r:id="rId36" xr:uid="{CE808D58-61B9-423B-AD81-E68A94792CFB}"/>
     <hyperlink ref="B26" r:id="rId37" xr:uid="{F1297A01-61E3-4759-9D5D-D9A6F9BCB77E}"/>
     <hyperlink ref="B23" r:id="rId38" xr:uid="{C745FACC-7FAC-461E-90D4-9BC0A4025913}"/>
-    <hyperlink ref="B59" r:id="rId39" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="B60" r:id="rId39" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
     <hyperlink ref="B41" r:id="rId40" xr:uid="{19683C75-D4BA-4207-8A88-14E281FC0EF3}"/>
     <hyperlink ref="B21" r:id="rId41" xr:uid="{90E3F36C-96B8-4969-BD97-8904E85B3EC2}"/>
-    <hyperlink ref="B55" r:id="rId42" xr:uid="{C93BA389-85D0-4EED-A95D-B84989BC0704}"/>
+    <hyperlink ref="B56" r:id="rId42" xr:uid="{C93BA389-85D0-4EED-A95D-B84989BC0704}"/>
+    <hyperlink ref="B42" r:id="rId43" xr:uid="{8556A3F1-43A8-4BAA-A91F-1991C3AFC98E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added Petition for rule to show cause to forms spreadsheet
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ilao_docassemble_easy_forms.xlsx
+++ b/docassemble/ILAO/data/sources/ilao_docassemble_easy_forms.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VivianM\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E111C3E7-F726-4DB1-BB52-B86D00C04FF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5734EC5F-EEA6-4BDD-A4AD-8FC53F1C1D64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="122">
   <si>
     <t>name</t>
   </si>
@@ -385,6 +385,12 @@
   </si>
   <si>
     <t>https://www.illinoislegalaid.org/legal-information/request-personal-property-left-inside-repossessed-car</t>
+  </si>
+  <si>
+    <t>Petition for rule to show cause - Family law cases</t>
+  </si>
+  <si>
+    <t>https://www.illinoislegalaid.org/legal-information/petition-rule-show-cause-family-law-cases</t>
   </si>
 </sst>
 </file>
@@ -747,7 +753,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B60"/>
+  <dimension ref="A1:B61"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="49.77734375" customWidth="1"/>
@@ -1028,209 +1034,217 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>42</v>
+        <v>120</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>43</v>
+        <v>121</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>65</v>
+        <v>47</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>112</v>
+        <v>63</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>113</v>
+        <v>65</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>100</v>
+        <v>118</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>16</v>
+        <v>119</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>79</v>
+        <v>16</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>99</v>
+        <v>79</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>27</v>
+        <v>98</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>28</v>
+        <v>99</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>74</v>
+        <v>27</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>9</v>
+        <v>68</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>8</v>
+        <v>69</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>61</v>
+        <v>9</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>60</v>
+        <v>8</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>14</v>
+        <v>76</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>15</v>
+        <v>77</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>116</v>
+        <v>34</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>117</v>
+        <v>35</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>96</v>
+        <v>116</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>97</v>
+        <v>117</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>81</v>
+        <v>102</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
+        <v>78</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
         <v>107</v>
       </c>
-      <c r="B60" s="1" t="s">
+      <c r="B61" s="1" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1242,46 +1256,47 @@
     <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="B20" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="B17" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="B50" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="B51" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
     <hyperlink ref="B24" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="B54" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="B43" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="B55" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="B44" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
     <hyperlink ref="B12" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
     <hyperlink ref="B13" r:id="rId9" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
     <hyperlink ref="B14" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="B46" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="B47" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
     <hyperlink ref="B25" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
     <hyperlink ref="B28" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="B55" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="B37" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="B38" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="B36" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="B35" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="B56" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="B38" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="B39" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="B37" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="B36" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
     <hyperlink ref="B32" r:id="rId19" xr:uid="{E91D49D0-8A8A-49A5-B571-1E3A551885E4}"/>
     <hyperlink ref="B30" r:id="rId20" xr:uid="{5EB32812-DDAD-43E1-BEC1-0E8706BB78F8}"/>
     <hyperlink ref="B4" r:id="rId21" xr:uid="{A23C6535-E02D-4241-B7AA-C698CCDB6D31}"/>
     <hyperlink ref="B16" r:id="rId22" xr:uid="{5B0358E0-6FC3-4AF8-8E25-62EBF7059C1A}"/>
-    <hyperlink ref="B51" r:id="rId23" xr:uid="{1BD2E9FF-F69E-4E59-ACA9-BD41D2D4AE94}"/>
-    <hyperlink ref="B40" r:id="rId24" xr:uid="{620FD2E8-C9D1-4C14-8ED5-17B01AA5DA33}"/>
-    <hyperlink ref="B48" r:id="rId25" xr:uid="{226D490B-4537-4CB5-95DA-F750E9A0919D}"/>
-    <hyperlink ref="B52" r:id="rId26" xr:uid="{285D1364-5954-4A82-B493-EE664C0786D1}"/>
-    <hyperlink ref="B49" r:id="rId27" xr:uid="{BD0F8AFC-EDD1-4D31-AD59-8FAD5E6F7758}"/>
+    <hyperlink ref="B52" r:id="rId23" xr:uid="{1BD2E9FF-F69E-4E59-ACA9-BD41D2D4AE94}"/>
+    <hyperlink ref="B41" r:id="rId24" xr:uid="{620FD2E8-C9D1-4C14-8ED5-17B01AA5DA33}"/>
+    <hyperlink ref="B49" r:id="rId25" xr:uid="{226D490B-4537-4CB5-95DA-F750E9A0919D}"/>
+    <hyperlink ref="B53" r:id="rId26" xr:uid="{285D1364-5954-4A82-B493-EE664C0786D1}"/>
+    <hyperlink ref="B50" r:id="rId27" xr:uid="{BD0F8AFC-EDD1-4D31-AD59-8FAD5E6F7758}"/>
     <hyperlink ref="B8" r:id="rId28" xr:uid="{4EAFCFFB-67EF-4EA4-9306-448CF1D5D183}"/>
     <hyperlink ref="B22" r:id="rId29" xr:uid="{B1E55B86-EC01-47AD-AA8B-FA1792695821}"/>
-    <hyperlink ref="B44" r:id="rId30" xr:uid="{7A05A07A-CD46-49E0-8CAA-F7A2359DAFA6}"/>
-    <hyperlink ref="B59" r:id="rId31" xr:uid="{E8243C89-C7E6-4F98-8AB2-6F1F40304356}"/>
+    <hyperlink ref="B45" r:id="rId30" xr:uid="{7A05A07A-CD46-49E0-8CAA-F7A2359DAFA6}"/>
+    <hyperlink ref="B60" r:id="rId31" xr:uid="{E8243C89-C7E6-4F98-8AB2-6F1F40304356}"/>
     <hyperlink ref="B29" r:id="rId32" xr:uid="{A702F17D-AC4F-43CE-B44D-BF0EB0BA16F4}"/>
     <hyperlink ref="B9" r:id="rId33" xr:uid="{A79B08AB-EC87-4B3E-B1A5-DB2982598670}"/>
-    <hyperlink ref="B57" r:id="rId34" xr:uid="{ACF5336B-7760-4E17-AB95-B490DF08E9B7}"/>
-    <hyperlink ref="B45" r:id="rId35" xr:uid="{5B5F40DA-F64F-4CBD-A95F-EBC3267FFA16}"/>
-    <hyperlink ref="B58" r:id="rId36" xr:uid="{CE808D58-61B9-423B-AD81-E68A94792CFB}"/>
+    <hyperlink ref="B58" r:id="rId34" xr:uid="{ACF5336B-7760-4E17-AB95-B490DF08E9B7}"/>
+    <hyperlink ref="B46" r:id="rId35" xr:uid="{5B5F40DA-F64F-4CBD-A95F-EBC3267FFA16}"/>
+    <hyperlink ref="B59" r:id="rId36" xr:uid="{CE808D58-61B9-423B-AD81-E68A94792CFB}"/>
     <hyperlink ref="B26" r:id="rId37" xr:uid="{F1297A01-61E3-4759-9D5D-D9A6F9BCB77E}"/>
     <hyperlink ref="B23" r:id="rId38" xr:uid="{C745FACC-7FAC-461E-90D4-9BC0A4025913}"/>
-    <hyperlink ref="B60" r:id="rId39" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="B41" r:id="rId40" xr:uid="{19683C75-D4BA-4207-8A88-14E281FC0EF3}"/>
+    <hyperlink ref="B61" r:id="rId39" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="B42" r:id="rId40" xr:uid="{19683C75-D4BA-4207-8A88-14E281FC0EF3}"/>
     <hyperlink ref="B21" r:id="rId41" xr:uid="{90E3F36C-96B8-4969-BD97-8904E85B3EC2}"/>
-    <hyperlink ref="B56" r:id="rId42" xr:uid="{C93BA389-85D0-4EED-A95D-B84989BC0704}"/>
-    <hyperlink ref="B42" r:id="rId43" xr:uid="{8556A3F1-43A8-4BAA-A91F-1991C3AFC98E}"/>
+    <hyperlink ref="B57" r:id="rId42" xr:uid="{C93BA389-85D0-4EED-A95D-B84989BC0704}"/>
+    <hyperlink ref="B43" r:id="rId43" xr:uid="{8556A3F1-43A8-4BAA-A91F-1991C3AFC98E}"/>
+    <hyperlink ref="B35" r:id="rId44" xr:uid="{C4E8FA95-6903-4867-A6AC-9C1E8F6118C1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added expungement easy form to xlsx
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ilao_docassemble_easy_forms.xlsx
+++ b/docassemble/ILAO/data/sources/ilao_docassemble_easy_forms.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VivianM\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5734EC5F-EEA6-4BDD-A4AD-8FC53F1C1D64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C77BEEFB-9AD3-4B65-9779-7034BC9C9713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5340" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="124">
   <si>
     <t>name</t>
   </si>
@@ -391,6 +391,12 @@
   </si>
   <si>
     <t>https://www.illinoislegalaid.org/legal-information/petition-rule-show-cause-family-law-cases</t>
+  </si>
+  <si>
+    <t>https://www.illinoislegalaid.org/legal-information/criminal-record-expungement-or-sealing-request</t>
+  </si>
+  <si>
+    <t>Expunge or seal criminal records</t>
   </si>
 </sst>
 </file>
@@ -753,7 +759,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:B62"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="49.77734375" customWidth="1"/>
@@ -906,397 +912,405 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>54</v>
+        <v>123</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>3</v>
+        <v>54</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>6</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>114</v>
+        <v>3</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>115</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>114</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>73</v>
+        <v>115</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>110</v>
+        <v>72</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>111</v>
+        <v>73</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>10</v>
+        <v>110</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>11</v>
+        <v>111</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>106</v>
+        <v>30</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>105</v>
+        <v>32</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>25</v>
+        <v>106</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>83</v>
+        <v>31</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>82</v>
+        <v>33</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>50</v>
+        <v>83</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>51</v>
+        <v>82</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>86</v>
+        <v>48</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>87</v>
+        <v>49</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>44</v>
+        <v>86</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>45</v>
+        <v>87</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>120</v>
+        <v>44</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>121</v>
+        <v>45</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>42</v>
+        <v>120</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>43</v>
+        <v>121</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>65</v>
+        <v>47</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>112</v>
+        <v>63</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>113</v>
+        <v>65</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>100</v>
+        <v>118</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>16</v>
+        <v>119</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>79</v>
+        <v>16</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>99</v>
+        <v>79</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>27</v>
+        <v>98</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>28</v>
+        <v>99</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>74</v>
+        <v>27</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>9</v>
+        <v>68</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>8</v>
+        <v>69</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>61</v>
+        <v>9</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>60</v>
+        <v>8</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>14</v>
+        <v>76</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>15</v>
+        <v>77</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>116</v>
+        <v>34</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>117</v>
+        <v>35</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>96</v>
+        <v>116</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>97</v>
+        <v>117</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>81</v>
+        <v>102</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
+        <v>78</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
         <v>107</v>
       </c>
-      <c r="B61" s="1" t="s">
+      <c r="B62" s="1" t="s">
         <v>29</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B20">
-    <sortCondition ref="A2:A20"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B21">
+    <sortCondition ref="A2:A21"/>
   </sortState>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="B20" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="B21" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="B17" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="B51" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="B24" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="B55" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="B44" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="B52" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="B25" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="B56" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="B45" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
     <hyperlink ref="B12" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
     <hyperlink ref="B13" r:id="rId9" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
     <hyperlink ref="B14" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="B47" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="B25" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="B28" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="B56" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="B38" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="B39" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="B37" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="B36" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="B32" r:id="rId19" xr:uid="{E91D49D0-8A8A-49A5-B571-1E3A551885E4}"/>
-    <hyperlink ref="B30" r:id="rId20" xr:uid="{5EB32812-DDAD-43E1-BEC1-0E8706BB78F8}"/>
+    <hyperlink ref="B48" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="B26" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="B29" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="B57" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="B39" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="B40" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="B38" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="B37" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="B33" r:id="rId19" xr:uid="{E91D49D0-8A8A-49A5-B571-1E3A551885E4}"/>
+    <hyperlink ref="B31" r:id="rId20" xr:uid="{5EB32812-DDAD-43E1-BEC1-0E8706BB78F8}"/>
     <hyperlink ref="B4" r:id="rId21" xr:uid="{A23C6535-E02D-4241-B7AA-C698CCDB6D31}"/>
     <hyperlink ref="B16" r:id="rId22" xr:uid="{5B0358E0-6FC3-4AF8-8E25-62EBF7059C1A}"/>
-    <hyperlink ref="B52" r:id="rId23" xr:uid="{1BD2E9FF-F69E-4E59-ACA9-BD41D2D4AE94}"/>
-    <hyperlink ref="B41" r:id="rId24" xr:uid="{620FD2E8-C9D1-4C14-8ED5-17B01AA5DA33}"/>
-    <hyperlink ref="B49" r:id="rId25" xr:uid="{226D490B-4537-4CB5-95DA-F750E9A0919D}"/>
-    <hyperlink ref="B53" r:id="rId26" xr:uid="{285D1364-5954-4A82-B493-EE664C0786D1}"/>
-    <hyperlink ref="B50" r:id="rId27" xr:uid="{BD0F8AFC-EDD1-4D31-AD59-8FAD5E6F7758}"/>
+    <hyperlink ref="B53" r:id="rId23" xr:uid="{1BD2E9FF-F69E-4E59-ACA9-BD41D2D4AE94}"/>
+    <hyperlink ref="B42" r:id="rId24" xr:uid="{620FD2E8-C9D1-4C14-8ED5-17B01AA5DA33}"/>
+    <hyperlink ref="B50" r:id="rId25" xr:uid="{226D490B-4537-4CB5-95DA-F750E9A0919D}"/>
+    <hyperlink ref="B54" r:id="rId26" xr:uid="{285D1364-5954-4A82-B493-EE664C0786D1}"/>
+    <hyperlink ref="B51" r:id="rId27" xr:uid="{BD0F8AFC-EDD1-4D31-AD59-8FAD5E6F7758}"/>
     <hyperlink ref="B8" r:id="rId28" xr:uid="{4EAFCFFB-67EF-4EA4-9306-448CF1D5D183}"/>
-    <hyperlink ref="B22" r:id="rId29" xr:uid="{B1E55B86-EC01-47AD-AA8B-FA1792695821}"/>
-    <hyperlink ref="B45" r:id="rId30" xr:uid="{7A05A07A-CD46-49E0-8CAA-F7A2359DAFA6}"/>
-    <hyperlink ref="B60" r:id="rId31" xr:uid="{E8243C89-C7E6-4F98-8AB2-6F1F40304356}"/>
-    <hyperlink ref="B29" r:id="rId32" xr:uid="{A702F17D-AC4F-43CE-B44D-BF0EB0BA16F4}"/>
+    <hyperlink ref="B23" r:id="rId29" xr:uid="{B1E55B86-EC01-47AD-AA8B-FA1792695821}"/>
+    <hyperlink ref="B46" r:id="rId30" xr:uid="{7A05A07A-CD46-49E0-8CAA-F7A2359DAFA6}"/>
+    <hyperlink ref="B61" r:id="rId31" xr:uid="{E8243C89-C7E6-4F98-8AB2-6F1F40304356}"/>
+    <hyperlink ref="B30" r:id="rId32" xr:uid="{A702F17D-AC4F-43CE-B44D-BF0EB0BA16F4}"/>
     <hyperlink ref="B9" r:id="rId33" xr:uid="{A79B08AB-EC87-4B3E-B1A5-DB2982598670}"/>
-    <hyperlink ref="B58" r:id="rId34" xr:uid="{ACF5336B-7760-4E17-AB95-B490DF08E9B7}"/>
-    <hyperlink ref="B46" r:id="rId35" xr:uid="{5B5F40DA-F64F-4CBD-A95F-EBC3267FFA16}"/>
-    <hyperlink ref="B59" r:id="rId36" xr:uid="{CE808D58-61B9-423B-AD81-E68A94792CFB}"/>
-    <hyperlink ref="B26" r:id="rId37" xr:uid="{F1297A01-61E3-4759-9D5D-D9A6F9BCB77E}"/>
-    <hyperlink ref="B23" r:id="rId38" xr:uid="{C745FACC-7FAC-461E-90D4-9BC0A4025913}"/>
-    <hyperlink ref="B61" r:id="rId39" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="B42" r:id="rId40" xr:uid="{19683C75-D4BA-4207-8A88-14E281FC0EF3}"/>
-    <hyperlink ref="B21" r:id="rId41" xr:uid="{90E3F36C-96B8-4969-BD97-8904E85B3EC2}"/>
-    <hyperlink ref="B57" r:id="rId42" xr:uid="{C93BA389-85D0-4EED-A95D-B84989BC0704}"/>
-    <hyperlink ref="B43" r:id="rId43" xr:uid="{8556A3F1-43A8-4BAA-A91F-1991C3AFC98E}"/>
-    <hyperlink ref="B35" r:id="rId44" xr:uid="{C4E8FA95-6903-4867-A6AC-9C1E8F6118C1}"/>
+    <hyperlink ref="B59" r:id="rId34" xr:uid="{ACF5336B-7760-4E17-AB95-B490DF08E9B7}"/>
+    <hyperlink ref="B47" r:id="rId35" xr:uid="{5B5F40DA-F64F-4CBD-A95F-EBC3267FFA16}"/>
+    <hyperlink ref="B60" r:id="rId36" xr:uid="{CE808D58-61B9-423B-AD81-E68A94792CFB}"/>
+    <hyperlink ref="B27" r:id="rId37" xr:uid="{F1297A01-61E3-4759-9D5D-D9A6F9BCB77E}"/>
+    <hyperlink ref="B24" r:id="rId38" xr:uid="{C745FACC-7FAC-461E-90D4-9BC0A4025913}"/>
+    <hyperlink ref="B62" r:id="rId39" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="B43" r:id="rId40" xr:uid="{19683C75-D4BA-4207-8A88-14E281FC0EF3}"/>
+    <hyperlink ref="B22" r:id="rId41" xr:uid="{90E3F36C-96B8-4969-BD97-8904E85B3EC2}"/>
+    <hyperlink ref="B58" r:id="rId42" xr:uid="{C93BA389-85D0-4EED-A95D-B84989BC0704}"/>
+    <hyperlink ref="B44" r:id="rId43" xr:uid="{8556A3F1-43A8-4BAA-A91F-1991C3AFC98E}"/>
+    <hyperlink ref="B36" r:id="rId44" xr:uid="{C4E8FA95-6903-4867-A6AC-9C1E8F6118C1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
updated default foreclosure url in xlsx
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ilao_docassemble_easy_forms.xlsx
+++ b/docassemble/ILAO/data/sources/ilao_docassemble_easy_forms.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C77BEEFB-9AD3-4B65-9779-7034BC9C9713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEA27B28-853D-4604-BB22-676AD91A3581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5340" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -333,9 +333,6 @@
     <t>Vacate a default judgment of foreclosure</t>
   </si>
   <si>
-    <t>https://easyforms.illinoislegalaid.org/start/VacateDefaultForeclosure/vacate_default_foreclosure</t>
-  </si>
-  <si>
     <t>Emergency Motion to Claim Exemption</t>
   </si>
   <si>
@@ -397,6 +394,9 @@
   </si>
   <si>
     <t>Expunge or seal criminal records</t>
+  </si>
+  <si>
+    <t>https://www.illinoislegalaid.org/legal-information/vacate-default-judgment-foreclosure</t>
   </si>
 </sst>
 </file>
@@ -816,10 +816,10 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>107</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -880,10 +880,10 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
+        <v>102</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
@@ -912,10 +912,10 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
@@ -936,10 +936,10 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
+        <v>113</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
@@ -952,10 +952,10 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
+        <v>109</v>
+      </c>
+      <c r="B24" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
@@ -976,10 +976,10 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
@@ -1048,10 +1048,10 @@
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
+        <v>119</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
@@ -1104,18 +1104,18 @@
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
+        <v>111</v>
+      </c>
+      <c r="B43" s="1" t="s">
         <v>112</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
+        <v>117</v>
+      </c>
+      <c r="B44" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
@@ -1224,10 +1224,10 @@
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
+        <v>115</v>
+      </c>
+      <c r="B58" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="B58" s="1" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
@@ -1243,7 +1243,7 @@
         <v>101</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>102</v>
+        <v>123</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.3">
@@ -1256,7 +1256,7 @@
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B62" s="1" t="s">
         <v>29</v>
@@ -1302,15 +1302,14 @@
     <hyperlink ref="B9" r:id="rId33" xr:uid="{A79B08AB-EC87-4B3E-B1A5-DB2982598670}"/>
     <hyperlink ref="B59" r:id="rId34" xr:uid="{ACF5336B-7760-4E17-AB95-B490DF08E9B7}"/>
     <hyperlink ref="B47" r:id="rId35" xr:uid="{5B5F40DA-F64F-4CBD-A95F-EBC3267FFA16}"/>
-    <hyperlink ref="B60" r:id="rId36" xr:uid="{CE808D58-61B9-423B-AD81-E68A94792CFB}"/>
-    <hyperlink ref="B27" r:id="rId37" xr:uid="{F1297A01-61E3-4759-9D5D-D9A6F9BCB77E}"/>
-    <hyperlink ref="B24" r:id="rId38" xr:uid="{C745FACC-7FAC-461E-90D4-9BC0A4025913}"/>
-    <hyperlink ref="B62" r:id="rId39" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="B43" r:id="rId40" xr:uid="{19683C75-D4BA-4207-8A88-14E281FC0EF3}"/>
-    <hyperlink ref="B22" r:id="rId41" xr:uid="{90E3F36C-96B8-4969-BD97-8904E85B3EC2}"/>
-    <hyperlink ref="B58" r:id="rId42" xr:uid="{C93BA389-85D0-4EED-A95D-B84989BC0704}"/>
-    <hyperlink ref="B44" r:id="rId43" xr:uid="{8556A3F1-43A8-4BAA-A91F-1991C3AFC98E}"/>
-    <hyperlink ref="B36" r:id="rId44" xr:uid="{C4E8FA95-6903-4867-A6AC-9C1E8F6118C1}"/>
+    <hyperlink ref="B27" r:id="rId36" xr:uid="{F1297A01-61E3-4759-9D5D-D9A6F9BCB77E}"/>
+    <hyperlink ref="B24" r:id="rId37" xr:uid="{C745FACC-7FAC-461E-90D4-9BC0A4025913}"/>
+    <hyperlink ref="B62" r:id="rId38" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="B43" r:id="rId39" xr:uid="{19683C75-D4BA-4207-8A88-14E281FC0EF3}"/>
+    <hyperlink ref="B22" r:id="rId40" xr:uid="{90E3F36C-96B8-4969-BD97-8904E85B3EC2}"/>
+    <hyperlink ref="B58" r:id="rId41" xr:uid="{C93BA389-85D0-4EED-A95D-B84989BC0704}"/>
+    <hyperlink ref="B44" r:id="rId42" xr:uid="{8556A3F1-43A8-4BAA-A91F-1991C3AFC98E}"/>
+    <hyperlink ref="B36" r:id="rId43" xr:uid="{C4E8FA95-6903-4867-A6AC-9C1E8F6118C1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>